<commit_message>
feat: completar catálogo — Limpieza·Cabin y Bonded Stores
Añade 52 productos nuevos (de 214 → 266 total):
- Limpieza·Cabin: 32 productos (químicos, utensilios, higiene personal)
- Bonded Stores: 20 productos (tabaco, cerveza, espirituosos, misceláneos)

Regenera plantilla Excel para reflejar las nuevas categorías completas.
El conteo PROVISION_PRODUCT_COUNT se actualiza automáticamente en la UI.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-provisiones.xlsx
+++ b/public/plantilla-provisiones.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="374">
   <si>
     <t>DE JESÚS SHIP SUPPLY</t>
   </si>
@@ -51,7 +51,7 @@
     <t>10</t>
   </si>
   <si>
-    <t>214</t>
+    <t>266</t>
   </si>
   <si>
     <t>24h</t>
@@ -324,12 +324,15 @@
     <t>Cleaning · Cabin</t>
   </si>
   <si>
-    <t>—</t>
+    <t>32 productos</t>
   </si>
   <si>
     <t>Bonded Stores</t>
   </si>
   <si>
+    <t>20 productos</t>
+  </si>
+  <si>
     <t>De Jesús Ship Supply  ·  djshipsupply.com  ·  info@djshipsupply.com  ·  Plantilla generada automáticamente</t>
   </si>
   <si>
@@ -1023,10 +1026,190 @@
     <t>CATEGORÍA  ·  09 / 10</t>
   </si>
   <si>
-    <t>Productos disponibles bajo solicitud. Indique sus necesidades en la hoja Resumen.</t>
+    <t>Bleach (liquid chlorine)</t>
+  </si>
+  <si>
+    <t>Ltrs</t>
+  </si>
+  <si>
+    <t>Multi-purpose cleaner</t>
+  </si>
+  <si>
+    <t>Bathroom cleaner / descaler</t>
+  </si>
+  <si>
+    <t>Btls</t>
+  </si>
+  <si>
+    <t>Dish soap / washing-up liquid</t>
+  </si>
+  <si>
+    <t>Floor cleaner / degreaser</t>
+  </si>
+  <si>
+    <t>Glass cleaner</t>
+  </si>
+  <si>
+    <t>Toilet bowl cleaner</t>
+  </si>
+  <si>
+    <t>Laundry detergent (powder)</t>
+  </si>
+  <si>
+    <t>Kgs</t>
+  </si>
+  <si>
+    <t>Laundry detergent (liquid)</t>
+  </si>
+  <si>
+    <t>Fabric softener</t>
+  </si>
+  <si>
+    <t>Air freshener spray</t>
+  </si>
+  <si>
+    <t>Pcs</t>
+  </si>
+  <si>
+    <t>Insecticide spray</t>
+  </si>
+  <si>
+    <t>Mop heads</t>
+  </si>
+  <si>
+    <t>Broom with dustpan</t>
+  </si>
+  <si>
+    <t>Scrubbing brushes</t>
+  </si>
+  <si>
+    <t>Sponges / scrubbing pads</t>
+  </si>
+  <si>
+    <t>Pack</t>
+  </si>
+  <si>
+    <t>Microfiber cloths</t>
+  </si>
+  <si>
+    <t>Rubber gloves</t>
+  </si>
+  <si>
+    <t>Pairs</t>
+  </si>
+  <si>
+    <t>Garbage bags (large 200L)</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t>Garbage bags (medium 100L)</t>
+  </si>
+  <si>
+    <t>Toilet paper</t>
+  </si>
+  <si>
+    <t>Paper towels / kitchen roll</t>
+  </si>
+  <si>
+    <t>Hand soap (bar)</t>
+  </si>
+  <si>
+    <t>Hand soap (liquid)</t>
+  </si>
+  <si>
+    <t>Shampoo</t>
+  </si>
+  <si>
+    <t>Body wash / shower gel</t>
+  </si>
+  <si>
+    <t>Conditioner</t>
+  </si>
+  <si>
+    <t>Toothpaste</t>
+  </si>
+  <si>
+    <t>Toothbrushes</t>
+  </si>
+  <si>
+    <t>Shaving cream</t>
+  </si>
+  <si>
+    <t>Disposable razors</t>
+  </si>
+  <si>
+    <t>Deodorant</t>
   </si>
   <si>
     <t>CATEGORÍA  ·  10 / 10</t>
+  </si>
+  <si>
+    <t>Cigarettes (Marlboro)</t>
+  </si>
+  <si>
+    <t>Carton</t>
+  </si>
+  <si>
+    <t>Cigarettes (Winston)</t>
+  </si>
+  <si>
+    <t>Cigarettes (L&amp;M)</t>
+  </si>
+  <si>
+    <t>Cigarettes (Camel)</t>
+  </si>
+  <si>
+    <t>Rolling tobacco</t>
+  </si>
+  <si>
+    <t>Cigars</t>
+  </si>
+  <si>
+    <t>Beer (Presidente)</t>
+  </si>
+  <si>
+    <t>Case</t>
+  </si>
+  <si>
+    <t>Beer (Heineken)</t>
+  </si>
+  <si>
+    <t>Beer (Corona)</t>
+  </si>
+  <si>
+    <t>Beer (Budweiser)</t>
+  </si>
+  <si>
+    <t>Rum (Barceló añejo)</t>
+  </si>
+  <si>
+    <t>Rum (Brugal extra viejo)</t>
+  </si>
+  <si>
+    <t>Whisky (Johnnie Walker Red)</t>
+  </si>
+  <si>
+    <t>Whisky (Johnnie Walker Black)</t>
+  </si>
+  <si>
+    <t>Whisky (Jack Daniel's)</t>
+  </si>
+  <si>
+    <t>Vodka (Absolut)</t>
+  </si>
+  <si>
+    <t>Assorted chocolates</t>
+  </si>
+  <si>
+    <t>Assorted candy / sweets</t>
+  </si>
+  <si>
+    <t>Playing cards</t>
+  </si>
+  <si>
+    <t>Cigarette lighters</t>
   </si>
   <si>
     <t>RESUMEN  /  SUMMARY</t>
@@ -1501,7 +1684,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1685,9 +1868,6 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -2346,12 +2526,12 @@
         <v>61</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B31" s="38"/>
       <c r="C31" s="38"/>
@@ -2388,7 +2568,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2404,7 +2584,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -2451,50 +2631,457 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="62" t="s">
-        <v>293</v>
-      </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="43">
+        <v>1</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>294</v>
+      </c>
+      <c r="C8" s="45"/>
+      <c r="D8" s="46" t="s">
+        <v>295</v>
+      </c>
+      <c r="E8" s="47"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="48">
+        <v>2</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>296</v>
+      </c>
+      <c r="C9" s="45"/>
+      <c r="D9" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="E9" s="51"/>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-    </row>
-    <row r="12" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
+      <c r="A10" s="43">
+        <v>3</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E10" s="47"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="48">
+        <v>4</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>299</v>
+      </c>
+      <c r="C11" s="45"/>
+      <c r="D11" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="E11" s="51"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="43">
+        <v>5</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>300</v>
+      </c>
+      <c r="C12" s="45"/>
+      <c r="D12" s="46" t="s">
+        <v>295</v>
+      </c>
+      <c r="E12" s="47"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="48">
+        <v>6</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>301</v>
+      </c>
+      <c r="C13" s="45"/>
+      <c r="D13" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E13" s="51"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="43">
+        <v>7</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>302</v>
+      </c>
+      <c r="C14" s="45"/>
+      <c r="D14" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E14" s="47"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="48">
+        <v>8</v>
+      </c>
+      <c r="B15" s="49" t="s">
+        <v>303</v>
+      </c>
+      <c r="C15" s="45"/>
+      <c r="D15" s="50" t="s">
+        <v>304</v>
+      </c>
+      <c r="E15" s="51"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="43">
+        <v>9</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>305</v>
+      </c>
+      <c r="C16" s="45"/>
+      <c r="D16" s="46" t="s">
+        <v>295</v>
+      </c>
+      <c r="E16" s="47"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="48">
+        <v>10</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="C17" s="45"/>
+      <c r="D17" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="E17" s="51"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="43">
+        <v>11</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>307</v>
+      </c>
+      <c r="C18" s="45"/>
+      <c r="D18" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E18" s="47"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="48">
+        <v>12</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>309</v>
+      </c>
+      <c r="C19" s="45"/>
+      <c r="D19" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E19" s="51"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="43">
+        <v>13</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>310</v>
+      </c>
+      <c r="C20" s="45"/>
+      <c r="D20" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E20" s="47"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="48">
+        <v>14</v>
+      </c>
+      <c r="B21" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="C21" s="45"/>
+      <c r="D21" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E21" s="51"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="43">
+        <v>15</v>
+      </c>
+      <c r="B22" s="44" t="s">
+        <v>312</v>
+      </c>
+      <c r="C22" s="45"/>
+      <c r="D22" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E22" s="47"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="48">
+        <v>16</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="C23" s="45"/>
+      <c r="D23" s="50" t="s">
+        <v>314</v>
+      </c>
+      <c r="E23" s="51"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="43">
+        <v>17</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>315</v>
+      </c>
+      <c r="C24" s="45"/>
+      <c r="D24" s="46" t="s">
+        <v>314</v>
+      </c>
+      <c r="E24" s="47"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="48">
+        <v>18</v>
+      </c>
+      <c r="B25" s="49" t="s">
+        <v>316</v>
+      </c>
+      <c r="C25" s="45"/>
+      <c r="D25" s="50" t="s">
+        <v>317</v>
+      </c>
+      <c r="E25" s="51"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="43">
+        <v>19</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>318</v>
+      </c>
+      <c r="C26" s="45"/>
+      <c r="D26" s="46" t="s">
+        <v>319</v>
+      </c>
+      <c r="E26" s="47"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="48">
+        <v>20</v>
+      </c>
+      <c r="B27" s="49" t="s">
+        <v>320</v>
+      </c>
+      <c r="C27" s="45"/>
+      <c r="D27" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="E27" s="51"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="43">
+        <v>21</v>
+      </c>
+      <c r="B28" s="44" t="s">
+        <v>321</v>
+      </c>
+      <c r="C28" s="45"/>
+      <c r="D28" s="46" t="s">
+        <v>319</v>
+      </c>
+      <c r="E28" s="47"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="48">
+        <v>22</v>
+      </c>
+      <c r="B29" s="49" t="s">
+        <v>322</v>
+      </c>
+      <c r="C29" s="45"/>
+      <c r="D29" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="E29" s="51"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="43">
+        <v>23</v>
+      </c>
+      <c r="B30" s="44" t="s">
+        <v>323</v>
+      </c>
+      <c r="C30" s="45"/>
+      <c r="D30" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E30" s="47"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="48">
+        <v>24</v>
+      </c>
+      <c r="B31" s="49" t="s">
+        <v>324</v>
+      </c>
+      <c r="C31" s="45"/>
+      <c r="D31" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E31" s="51"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="43">
+        <v>25</v>
+      </c>
+      <c r="B32" s="44" t="s">
+        <v>325</v>
+      </c>
+      <c r="C32" s="45"/>
+      <c r="D32" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E32" s="47"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="48">
+        <v>26</v>
+      </c>
+      <c r="B33" s="49" t="s">
+        <v>326</v>
+      </c>
+      <c r="C33" s="45"/>
+      <c r="D33" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E33" s="51"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="43">
+        <v>27</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>327</v>
+      </c>
+      <c r="C34" s="45"/>
+      <c r="D34" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E34" s="47"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="48">
+        <v>28</v>
+      </c>
+      <c r="B35" s="49" t="s">
+        <v>328</v>
+      </c>
+      <c r="C35" s="45"/>
+      <c r="D35" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E35" s="51"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="43">
+        <v>29</v>
+      </c>
+      <c r="B36" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="C36" s="45"/>
+      <c r="D36" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E36" s="47"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="48">
+        <v>30</v>
+      </c>
+      <c r="B37" s="49" t="s">
+        <v>330</v>
+      </c>
+      <c r="C37" s="45"/>
+      <c r="D37" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E37" s="51"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="43">
+        <v>31</v>
+      </c>
+      <c r="B38" s="44" t="s">
+        <v>331</v>
+      </c>
+      <c r="C38" s="45"/>
+      <c r="D38" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E38" s="47"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="58">
+        <v>32</v>
+      </c>
+      <c r="B39" s="59" t="s">
+        <v>332</v>
+      </c>
+      <c r="C39" s="54"/>
+      <c r="D39" s="60" t="s">
+        <v>308</v>
+      </c>
+      <c r="E39" s="61"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="57" t="s">
+        <v>106</v>
+      </c>
+      <c r="B41" s="57"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="57"/>
+    </row>
+    <row r="43" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A2:B2"/>
@@ -2503,10 +3090,17 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:E43"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showErrorMessage="1" errorStyle="warning" errorTitle="Cantidad no válida" error="Introduzca un número mayor o igual a 0." sqref="C10:C39">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showErrorMessage="1" errorStyle="warning" errorTitle="Cantidad no válida" error="Introduzca un número mayor o igual a 0." sqref="C8:C39">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2517,7 +3111,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2533,7 +3127,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>294</v>
+        <v>333</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -2580,50 +3174,301 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="62" t="s">
-        <v>293</v>
-      </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="43">
+        <v>1</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>334</v>
+      </c>
+      <c r="C8" s="45"/>
+      <c r="D8" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="E8" s="47"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="48">
+        <v>2</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>336</v>
+      </c>
+      <c r="C9" s="45"/>
+      <c r="D9" s="50" t="s">
+        <v>335</v>
+      </c>
+      <c r="E9" s="51"/>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-    </row>
-    <row r="12" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
+      <c r="A10" s="43">
+        <v>3</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>337</v>
+      </c>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="E10" s="47"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="48">
+        <v>4</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11" s="45"/>
+      <c r="D11" s="50" t="s">
+        <v>335</v>
+      </c>
+      <c r="E11" s="51"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="43">
+        <v>5</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>339</v>
+      </c>
+      <c r="C12" s="45"/>
+      <c r="D12" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E12" s="47"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="48">
+        <v>6</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>340</v>
+      </c>
+      <c r="C13" s="45"/>
+      <c r="D13" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E13" s="51"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="43">
+        <v>7</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>341</v>
+      </c>
+      <c r="C14" s="45"/>
+      <c r="D14" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="E14" s="47"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="48">
+        <v>8</v>
+      </c>
+      <c r="B15" s="49" t="s">
+        <v>343</v>
+      </c>
+      <c r="C15" s="45"/>
+      <c r="D15" s="50" t="s">
+        <v>342</v>
+      </c>
+      <c r="E15" s="51"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="43">
+        <v>9</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>344</v>
+      </c>
+      <c r="C16" s="45"/>
+      <c r="D16" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="E16" s="47"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="48">
+        <v>10</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>345</v>
+      </c>
+      <c r="C17" s="45"/>
+      <c r="D17" s="50" t="s">
+        <v>342</v>
+      </c>
+      <c r="E17" s="51"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="43">
+        <v>11</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>346</v>
+      </c>
+      <c r="C18" s="45"/>
+      <c r="D18" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E18" s="47"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="48">
+        <v>12</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>347</v>
+      </c>
+      <c r="C19" s="45"/>
+      <c r="D19" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E19" s="51"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="43">
+        <v>13</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>348</v>
+      </c>
+      <c r="C20" s="45"/>
+      <c r="D20" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E20" s="47"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="48">
+        <v>14</v>
+      </c>
+      <c r="B21" s="49" t="s">
+        <v>349</v>
+      </c>
+      <c r="C21" s="45"/>
+      <c r="D21" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E21" s="51"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="43">
+        <v>15</v>
+      </c>
+      <c r="B22" s="44" t="s">
+        <v>350</v>
+      </c>
+      <c r="C22" s="45"/>
+      <c r="D22" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="E22" s="47"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="48">
+        <v>16</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>351</v>
+      </c>
+      <c r="C23" s="45"/>
+      <c r="D23" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E23" s="51"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="43">
+        <v>17</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>352</v>
+      </c>
+      <c r="C24" s="45"/>
+      <c r="D24" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E24" s="47"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="48">
+        <v>18</v>
+      </c>
+      <c r="B25" s="49" t="s">
+        <v>353</v>
+      </c>
+      <c r="C25" s="45"/>
+      <c r="D25" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E25" s="51"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="43">
+        <v>19</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>354</v>
+      </c>
+      <c r="C26" s="45"/>
+      <c r="D26" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="E26" s="47"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="58">
+        <v>20</v>
+      </c>
+      <c r="B27" s="59" t="s">
+        <v>355</v>
+      </c>
+      <c r="C27" s="54"/>
+      <c r="D27" s="60" t="s">
+        <v>308</v>
+      </c>
+      <c r="E27" s="61"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="57" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" s="57"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+    </row>
+    <row r="31" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A2:B2"/>
@@ -2632,10 +3477,17 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A31:E31"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showErrorMessage="1" errorStyle="warning" errorTitle="Cantidad no válida" error="Introduzca un número mayor o igual a 0." sqref="C10:C27">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showErrorMessage="1" errorStyle="warning" errorTitle="Cantidad no válida" error="Introduzca un número mayor o igual a 0." sqref="C8:C27">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2654,15 +3506,15 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>295</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="63" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -2670,7 +3522,7 @@
       </c>
     </row>
     <row r="3" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="65" t="s">
+      <c r="A3" s="64" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -2679,169 +3531,169 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>296</v>
+        <v>357</v>
       </c>
       <c r="B4" s="7"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>297</v>
+        <v>358</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>298</v>
+        <v>359</v>
       </c>
       <c r="B7" s="15"/>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="66" t="s">
-        <v>299</v>
-      </c>
-      <c r="B8" s="67" t="s">
-        <v>70</v>
+      <c r="A8" s="65" t="s">
+        <v>360</v>
+      </c>
+      <c r="B8" s="66" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="68" t="s">
-        <v>300</v>
-      </c>
-      <c r="B9" s="69" t="s">
-        <v>70</v>
+      <c r="A9" s="67" t="s">
+        <v>361</v>
+      </c>
+      <c r="B9" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="68" t="s">
-        <v>301</v>
-      </c>
-      <c r="B10" s="70" t="s">
-        <v>70</v>
+      <c r="A10" s="67" t="s">
+        <v>362</v>
+      </c>
+      <c r="B10" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="68" t="s">
-        <v>302</v>
-      </c>
-      <c r="B11" s="69" t="s">
-        <v>70</v>
+      <c r="A11" s="67" t="s">
+        <v>363</v>
+      </c>
+      <c r="B11" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="68" t="s">
-        <v>303</v>
-      </c>
-      <c r="B12" s="70" t="s">
-        <v>70</v>
+      <c r="A12" s="67" t="s">
+        <v>364</v>
+      </c>
+      <c r="B12" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="68" t="s">
-        <v>304</v>
-      </c>
-      <c r="B13" s="69" t="s">
-        <v>70</v>
+      <c r="A13" s="67" t="s">
+        <v>365</v>
+      </c>
+      <c r="B13" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="68" t="s">
-        <v>305</v>
-      </c>
-      <c r="B14" s="70" t="s">
-        <v>70</v>
+      <c r="A14" s="67" t="s">
+        <v>366</v>
+      </c>
+      <c r="B14" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="68" t="s">
-        <v>306</v>
-      </c>
-      <c r="B15" s="69" t="s">
-        <v>70</v>
+      <c r="A15" s="67" t="s">
+        <v>367</v>
+      </c>
+      <c r="B15" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="68" t="s">
-        <v>307</v>
-      </c>
-      <c r="B16" s="70" t="s">
-        <v>70</v>
+      <c r="A16" s="67" t="s">
+        <v>368</v>
+      </c>
+      <c r="B16" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="68" t="s">
-        <v>308</v>
-      </c>
-      <c r="B17" s="69" t="s">
-        <v>70</v>
+      <c r="A17" s="67" t="s">
+        <v>369</v>
+      </c>
+      <c r="B17" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="68" t="s">
-        <v>309</v>
-      </c>
-      <c r="B18" s="70" t="s">
-        <v>70</v>
+      <c r="A18" s="67" t="s">
+        <v>370</v>
+      </c>
+      <c r="B18" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="68" t="s">
-        <v>310</v>
-      </c>
-      <c r="B19" s="69" t="s">
-        <v>70</v>
+      <c r="A19" s="67" t="s">
+        <v>371</v>
+      </c>
+      <c r="B19" s="68" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="71" t="s">
-        <v>311</v>
-      </c>
-      <c r="B20" s="72" t="s">
-        <v>70</v>
+      <c r="A20" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="B20" s="71" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>312</v>
+        <v>373</v>
       </c>
       <c r="B23" s="15"/>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="73" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="73"/>
+      <c r="A24" s="72" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="72"/>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="73"/>
-      <c r="B25" s="73"/>
+      <c r="A25" s="72"/>
+      <c r="B25" s="72"/>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="73"/>
-      <c r="B26" s="73"/>
+      <c r="A26" s="72"/>
+      <c r="B26" s="72"/>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="73"/>
-      <c r="B27" s="73"/>
+      <c r="A27" s="72"/>
+      <c r="B27" s="72"/>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="73"/>
-      <c r="B28" s="73"/>
+      <c r="A28" s="72"/>
+      <c r="B28" s="72"/>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="73"/>
-      <c r="B29" s="73"/>
+      <c r="A29" s="72"/>
+      <c r="B29" s="72"/>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="73"/>
-      <c r="B30" s="73"/>
+      <c r="A30" s="72"/>
+      <c r="B30" s="72"/>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="73"/>
-      <c r="B31" s="73"/>
+      <c r="A31" s="72"/>
+      <c r="B31" s="72"/>
     </row>
     <row r="34" ht="14" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B34" s="38"/>
     </row>
@@ -2880,7 +3732,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -2927,19 +3779,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2947,11 +3799,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -2960,11 +3812,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -2973,11 +3825,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -2986,11 +3838,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -2999,11 +3851,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -3012,11 +3864,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -3025,11 +3877,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -3038,11 +3890,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -3051,11 +3903,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -3064,11 +3916,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -3077,11 +3929,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C18" s="45"/>
       <c r="D18" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="47"/>
     </row>
@@ -3090,11 +3942,11 @@
         <v>12</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C19" s="45"/>
       <c r="D19" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E19" s="51"/>
     </row>
@@ -3103,11 +3955,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="47"/>
     </row>
@@ -3116,11 +3968,11 @@
         <v>14</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="51"/>
     </row>
@@ -3129,11 +3981,11 @@
         <v>15</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="47"/>
     </row>
@@ -3142,11 +3994,11 @@
         <v>16</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E23" s="51"/>
     </row>
@@ -3155,11 +4007,11 @@
         <v>17</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="47"/>
     </row>
@@ -3168,11 +4020,11 @@
         <v>18</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" s="51"/>
     </row>
@@ -3181,11 +4033,11 @@
         <v>19</v>
       </c>
       <c r="B26" s="44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E26" s="47"/>
     </row>
@@ -3194,11 +4046,11 @@
         <v>20</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E27" s="51"/>
     </row>
@@ -3207,11 +4059,11 @@
         <v>21</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E28" s="47"/>
     </row>
@@ -3220,11 +4072,11 @@
         <v>22</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E29" s="51"/>
     </row>
@@ -3233,11 +4085,11 @@
         <v>23</v>
       </c>
       <c r="B30" s="44" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E30" s="47"/>
     </row>
@@ -3246,11 +4098,11 @@
         <v>24</v>
       </c>
       <c r="B31" s="49" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C31" s="45"/>
       <c r="D31" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E31" s="51"/>
     </row>
@@ -3259,11 +4111,11 @@
         <v>25</v>
       </c>
       <c r="B32" s="44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E32" s="47"/>
     </row>
@@ -3272,11 +4124,11 @@
         <v>26</v>
       </c>
       <c r="B33" s="49" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C33" s="45"/>
       <c r="D33" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E33" s="51"/>
     </row>
@@ -3285,11 +4137,11 @@
         <v>27</v>
       </c>
       <c r="B34" s="44" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C34" s="45"/>
       <c r="D34" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E34" s="47"/>
     </row>
@@ -3298,11 +4150,11 @@
         <v>28</v>
       </c>
       <c r="B35" s="49" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C35" s="45"/>
       <c r="D35" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E35" s="51"/>
     </row>
@@ -3311,11 +4163,11 @@
         <v>29</v>
       </c>
       <c r="B36" s="44" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C36" s="45"/>
       <c r="D36" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E36" s="47"/>
     </row>
@@ -3324,11 +4176,11 @@
         <v>30</v>
       </c>
       <c r="B37" s="49" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C37" s="45"/>
       <c r="D37" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E37" s="51"/>
     </row>
@@ -3337,11 +4189,11 @@
         <v>31</v>
       </c>
       <c r="B38" s="44" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C38" s="45"/>
       <c r="D38" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E38" s="47"/>
     </row>
@@ -3350,11 +4202,11 @@
         <v>32</v>
       </c>
       <c r="B39" s="49" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39" s="45"/>
       <c r="D39" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E39" s="51"/>
     </row>
@@ -3363,11 +4215,11 @@
         <v>33</v>
       </c>
       <c r="B40" s="44" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C40" s="45"/>
       <c r="D40" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E40" s="47"/>
     </row>
@@ -3376,11 +4228,11 @@
         <v>34</v>
       </c>
       <c r="B41" s="49" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C41" s="45"/>
       <c r="D41" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E41" s="51"/>
     </row>
@@ -3389,17 +4241,17 @@
         <v>35</v>
       </c>
       <c r="B42" s="53" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C42" s="54"/>
       <c r="D42" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E42" s="56"/>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B44" s="57"/>
       <c r="C44" s="57"/>
@@ -3408,7 +4260,7 @@
     </row>
     <row r="46" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B46" s="38"/>
       <c r="C46" s="38"/>
@@ -3462,7 +4314,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -3509,19 +4361,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3529,11 +4381,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -3542,11 +4394,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -3555,11 +4407,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -3568,11 +4420,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -3581,11 +4433,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -3594,11 +4446,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -3607,11 +4459,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -3620,11 +4472,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -3633,11 +4485,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -3646,11 +4498,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -3659,17 +4511,17 @@
         <v>11</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C18" s="54"/>
       <c r="D18" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="56"/>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B20" s="57"/>
       <c r="C20" s="57"/>
@@ -3678,7 +4530,7 @@
     </row>
     <row r="22" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B22" s="38"/>
       <c r="C22" s="38"/>
@@ -3732,7 +4584,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -3779,19 +4631,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3799,11 +4651,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -3812,11 +4664,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -3825,11 +4677,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -3838,11 +4690,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -3851,11 +4703,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -3864,11 +4716,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -3877,11 +4729,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -3890,11 +4742,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -3903,11 +4755,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -3916,11 +4768,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -3929,11 +4781,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C18" s="45"/>
       <c r="D18" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="47"/>
     </row>
@@ -3942,17 +4794,17 @@
         <v>12</v>
       </c>
       <c r="B19" s="59" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C19" s="54"/>
       <c r="D19" s="60" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E19" s="61"/>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B21" s="57"/>
       <c r="C21" s="57"/>
@@ -3961,7 +4813,7 @@
     </row>
     <row r="23" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B23" s="38"/>
       <c r="C23" s="38"/>
@@ -4015,7 +4867,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -4062,19 +4914,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4082,11 +4934,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -4095,11 +4947,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -4108,11 +4960,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -4121,11 +4973,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -4134,11 +4986,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -4147,11 +4999,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -4160,11 +5012,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -4173,11 +5025,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -4186,11 +5038,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -4199,11 +5051,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -4212,11 +5064,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C18" s="45"/>
       <c r="D18" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="47"/>
     </row>
@@ -4225,11 +5077,11 @@
         <v>12</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C19" s="45"/>
       <c r="D19" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E19" s="51"/>
     </row>
@@ -4238,11 +5090,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="47"/>
     </row>
@@ -4251,11 +5103,11 @@
         <v>14</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="51"/>
     </row>
@@ -4264,11 +5116,11 @@
         <v>15</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="47"/>
     </row>
@@ -4277,11 +5129,11 @@
         <v>16</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E23" s="51"/>
     </row>
@@ -4290,11 +5142,11 @@
         <v>17</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="47"/>
     </row>
@@ -4303,11 +5155,11 @@
         <v>18</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" s="51"/>
     </row>
@@ -4316,17 +5168,17 @@
         <v>19</v>
       </c>
       <c r="B26" s="53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C26" s="54"/>
       <c r="D26" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E26" s="56"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B28" s="57"/>
       <c r="C28" s="57"/>
@@ -4335,7 +5187,7 @@
     </row>
     <row r="30" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B30" s="38"/>
       <c r="C30" s="38"/>
@@ -4389,7 +5241,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -4436,19 +5288,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4456,11 +5308,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -4469,11 +5321,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -4482,11 +5334,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -4495,11 +5347,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -4508,11 +5360,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -4521,11 +5373,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -4534,17 +5386,17 @@
         <v>7</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C14" s="54"/>
       <c r="D14" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="56"/>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B16" s="57"/>
       <c r="C16" s="57"/>
@@ -4553,7 +5405,7 @@
     </row>
     <row r="18" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B18" s="38"/>
       <c r="C18" s="38"/>
@@ -4607,7 +5459,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -4654,19 +5506,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4674,11 +5526,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -4687,11 +5539,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -4700,11 +5552,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -4713,11 +5565,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -4726,11 +5578,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -4739,11 +5591,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -4752,11 +5604,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -4765,11 +5617,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -4778,11 +5630,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -4791,11 +5643,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -4804,11 +5656,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C18" s="45"/>
       <c r="D18" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="47"/>
     </row>
@@ -4817,11 +5669,11 @@
         <v>12</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" s="45"/>
       <c r="D19" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E19" s="51"/>
     </row>
@@ -4830,11 +5682,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="47"/>
     </row>
@@ -4843,11 +5695,11 @@
         <v>14</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="51"/>
     </row>
@@ -4856,11 +5708,11 @@
         <v>15</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="47"/>
     </row>
@@ -4869,11 +5721,11 @@
         <v>16</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E23" s="51"/>
     </row>
@@ -4882,17 +5734,17 @@
         <v>17</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C24" s="54"/>
       <c r="D24" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="56"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B26" s="57"/>
       <c r="C26" s="57"/>
@@ -4901,7 +5753,7 @@
     </row>
     <row r="28" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B28" s="38"/>
       <c r="C28" s="38"/>
@@ -4955,7 +5807,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -5002,19 +5854,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5022,11 +5874,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -5035,11 +5887,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -5048,11 +5900,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -5061,11 +5913,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -5074,11 +5926,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -5087,11 +5939,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -5100,11 +5952,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -5113,11 +5965,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -5126,11 +5978,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -5139,11 +5991,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -5152,17 +6004,17 @@
         <v>11</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C18" s="54"/>
       <c r="D18" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="56"/>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B20" s="57"/>
       <c r="C20" s="57"/>
@@ -5171,7 +6023,7 @@
     </row>
     <row r="22" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B22" s="38"/>
       <c r="C22" s="38"/>
@@ -5225,7 +6077,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -5272,19 +6124,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5292,11 +6144,11 @@
         <v>1</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="47"/>
     </row>
@@ -5305,11 +6157,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" s="51"/>
     </row>
@@ -5318,11 +6170,11 @@
         <v>3</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="47"/>
     </row>
@@ -5331,11 +6183,11 @@
         <v>4</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="51"/>
     </row>
@@ -5344,11 +6196,11 @@
         <v>5</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="47"/>
     </row>
@@ -5357,11 +6209,11 @@
         <v>6</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -5370,11 +6222,11 @@
         <v>7</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="47"/>
     </row>
@@ -5383,11 +6235,11 @@
         <v>8</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="51"/>
     </row>
@@ -5396,11 +6248,11 @@
         <v>9</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C16" s="45"/>
       <c r="D16" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E16" s="47"/>
     </row>
@@ -5409,11 +6261,11 @@
         <v>10</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C17" s="45"/>
       <c r="D17" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="51"/>
     </row>
@@ -5422,11 +6274,11 @@
         <v>11</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C18" s="45"/>
       <c r="D18" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="47"/>
     </row>
@@ -5435,11 +6287,11 @@
         <v>12</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C19" s="45"/>
       <c r="D19" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E19" s="51"/>
     </row>
@@ -5448,11 +6300,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="47"/>
     </row>
@@ -5461,11 +6313,11 @@
         <v>14</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="51"/>
     </row>
@@ -5474,11 +6326,11 @@
         <v>15</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="47"/>
     </row>
@@ -5487,11 +6339,11 @@
         <v>16</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E23" s="51"/>
     </row>
@@ -5500,11 +6352,11 @@
         <v>17</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="47"/>
     </row>
@@ -5513,11 +6365,11 @@
         <v>18</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" s="51"/>
     </row>
@@ -5526,11 +6378,11 @@
         <v>19</v>
       </c>
       <c r="B26" s="44" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E26" s="47"/>
     </row>
@@ -5539,11 +6391,11 @@
         <v>20</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E27" s="51"/>
     </row>
@@ -5552,11 +6404,11 @@
         <v>21</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E28" s="47"/>
     </row>
@@ -5565,11 +6417,11 @@
         <v>22</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E29" s="51"/>
     </row>
@@ -5578,11 +6430,11 @@
         <v>23</v>
       </c>
       <c r="B30" s="44" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E30" s="47"/>
     </row>
@@ -5591,11 +6443,11 @@
         <v>24</v>
       </c>
       <c r="B31" s="49" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C31" s="45"/>
       <c r="D31" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E31" s="51"/>
     </row>
@@ -5604,11 +6456,11 @@
         <v>25</v>
       </c>
       <c r="B32" s="44" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E32" s="47"/>
     </row>
@@ -5617,11 +6469,11 @@
         <v>26</v>
       </c>
       <c r="B33" s="49" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C33" s="45"/>
       <c r="D33" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E33" s="51"/>
     </row>
@@ -5630,11 +6482,11 @@
         <v>27</v>
       </c>
       <c r="B34" s="44" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C34" s="45"/>
       <c r="D34" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E34" s="47"/>
     </row>
@@ -5643,11 +6495,11 @@
         <v>28</v>
       </c>
       <c r="B35" s="49" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C35" s="45"/>
       <c r="D35" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E35" s="51"/>
     </row>
@@ -5656,11 +6508,11 @@
         <v>29</v>
       </c>
       <c r="B36" s="44" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C36" s="45"/>
       <c r="D36" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E36" s="47"/>
     </row>
@@ -5669,11 +6521,11 @@
         <v>30</v>
       </c>
       <c r="B37" s="49" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C37" s="45"/>
       <c r="D37" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E37" s="51"/>
     </row>
@@ -5682,11 +6534,11 @@
         <v>31</v>
       </c>
       <c r="B38" s="44" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C38" s="45"/>
       <c r="D38" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E38" s="47"/>
     </row>
@@ -5695,11 +6547,11 @@
         <v>32</v>
       </c>
       <c r="B39" s="49" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C39" s="45"/>
       <c r="D39" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E39" s="51"/>
     </row>
@@ -5708,11 +6560,11 @@
         <v>33</v>
       </c>
       <c r="B40" s="44" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C40" s="45"/>
       <c r="D40" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E40" s="47"/>
     </row>
@@ -5721,11 +6573,11 @@
         <v>34</v>
       </c>
       <c r="B41" s="49" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C41" s="45"/>
       <c r="D41" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E41" s="51"/>
     </row>
@@ -5734,11 +6586,11 @@
         <v>35</v>
       </c>
       <c r="B42" s="44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C42" s="45"/>
       <c r="D42" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E42" s="47"/>
     </row>
@@ -5747,11 +6599,11 @@
         <v>36</v>
       </c>
       <c r="B43" s="49" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C43" s="45"/>
       <c r="D43" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E43" s="51"/>
     </row>
@@ -5760,11 +6612,11 @@
         <v>37</v>
       </c>
       <c r="B44" s="44" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C44" s="45"/>
       <c r="D44" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E44" s="47"/>
     </row>
@@ -5773,11 +6625,11 @@
         <v>38</v>
       </c>
       <c r="B45" s="49" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C45" s="45"/>
       <c r="D45" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E45" s="51"/>
     </row>
@@ -5786,11 +6638,11 @@
         <v>39</v>
       </c>
       <c r="B46" s="44" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C46" s="45"/>
       <c r="D46" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E46" s="47"/>
     </row>
@@ -5799,11 +6651,11 @@
         <v>40</v>
       </c>
       <c r="B47" s="49" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C47" s="45"/>
       <c r="D47" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E47" s="51"/>
     </row>
@@ -5812,11 +6664,11 @@
         <v>41</v>
       </c>
       <c r="B48" s="44" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C48" s="45"/>
       <c r="D48" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E48" s="47"/>
     </row>
@@ -5825,11 +6677,11 @@
         <v>42</v>
       </c>
       <c r="B49" s="49" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C49" s="45"/>
       <c r="D49" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E49" s="51"/>
     </row>
@@ -5838,11 +6690,11 @@
         <v>43</v>
       </c>
       <c r="B50" s="44" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C50" s="45"/>
       <c r="D50" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E50" s="47"/>
     </row>
@@ -5851,11 +6703,11 @@
         <v>44</v>
       </c>
       <c r="B51" s="49" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C51" s="45"/>
       <c r="D51" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E51" s="51"/>
     </row>
@@ -5864,11 +6716,11 @@
         <v>45</v>
       </c>
       <c r="B52" s="44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C52" s="45"/>
       <c r="D52" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E52" s="47"/>
     </row>
@@ -5877,11 +6729,11 @@
         <v>46</v>
       </c>
       <c r="B53" s="49" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C53" s="45"/>
       <c r="D53" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E53" s="51"/>
     </row>
@@ -5890,11 +6742,11 @@
         <v>47</v>
       </c>
       <c r="B54" s="44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C54" s="45"/>
       <c r="D54" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E54" s="47"/>
     </row>
@@ -5903,11 +6755,11 @@
         <v>48</v>
       </c>
       <c r="B55" s="49" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C55" s="45"/>
       <c r="D55" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E55" s="51"/>
     </row>
@@ -5916,11 +6768,11 @@
         <v>49</v>
       </c>
       <c r="B56" s="44" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C56" s="45"/>
       <c r="D56" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E56" s="47"/>
     </row>
@@ -5929,11 +6781,11 @@
         <v>50</v>
       </c>
       <c r="B57" s="49" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C57" s="45"/>
       <c r="D57" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E57" s="51"/>
     </row>
@@ -5942,11 +6794,11 @@
         <v>51</v>
       </c>
       <c r="B58" s="44" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C58" s="45"/>
       <c r="D58" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E58" s="47"/>
     </row>
@@ -5955,11 +6807,11 @@
         <v>52</v>
       </c>
       <c r="B59" s="49" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C59" s="45"/>
       <c r="D59" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E59" s="51"/>
     </row>
@@ -5968,11 +6820,11 @@
         <v>53</v>
       </c>
       <c r="B60" s="44" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C60" s="45"/>
       <c r="D60" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E60" s="47"/>
     </row>
@@ -5981,11 +6833,11 @@
         <v>54</v>
       </c>
       <c r="B61" s="49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C61" s="45"/>
       <c r="D61" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E61" s="51"/>
     </row>
@@ -5994,11 +6846,11 @@
         <v>55</v>
       </c>
       <c r="B62" s="44" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C62" s="45"/>
       <c r="D62" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E62" s="47"/>
     </row>
@@ -6007,11 +6859,11 @@
         <v>56</v>
       </c>
       <c r="B63" s="49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C63" s="45"/>
       <c r="D63" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E63" s="51"/>
     </row>
@@ -6020,11 +6872,11 @@
         <v>57</v>
       </c>
       <c r="B64" s="44" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C64" s="45"/>
       <c r="D64" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E64" s="47"/>
     </row>
@@ -6033,11 +6885,11 @@
         <v>58</v>
       </c>
       <c r="B65" s="49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C65" s="45"/>
       <c r="D65" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E65" s="51"/>
     </row>
@@ -6046,11 +6898,11 @@
         <v>59</v>
       </c>
       <c r="B66" s="44" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C66" s="45"/>
       <c r="D66" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E66" s="47"/>
     </row>
@@ -6059,11 +6911,11 @@
         <v>60</v>
       </c>
       <c r="B67" s="49" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C67" s="45"/>
       <c r="D67" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E67" s="51"/>
     </row>
@@ -6072,11 +6924,11 @@
         <v>61</v>
       </c>
       <c r="B68" s="44" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C68" s="45"/>
       <c r="D68" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E68" s="47"/>
     </row>
@@ -6085,11 +6937,11 @@
         <v>62</v>
       </c>
       <c r="B69" s="49" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C69" s="45"/>
       <c r="D69" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E69" s="51"/>
     </row>
@@ -6098,11 +6950,11 @@
         <v>63</v>
       </c>
       <c r="B70" s="44" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C70" s="45"/>
       <c r="D70" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E70" s="47"/>
     </row>
@@ -6111,11 +6963,11 @@
         <v>64</v>
       </c>
       <c r="B71" s="49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C71" s="45"/>
       <c r="D71" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E71" s="51"/>
     </row>
@@ -6124,11 +6976,11 @@
         <v>65</v>
       </c>
       <c r="B72" s="44" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C72" s="45"/>
       <c r="D72" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E72" s="47"/>
     </row>
@@ -6137,11 +6989,11 @@
         <v>66</v>
       </c>
       <c r="B73" s="49" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C73" s="45"/>
       <c r="D73" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E73" s="51"/>
     </row>
@@ -6150,11 +7002,11 @@
         <v>67</v>
       </c>
       <c r="B74" s="44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C74" s="45"/>
       <c r="D74" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E74" s="47"/>
     </row>
@@ -6163,11 +7015,11 @@
         <v>68</v>
       </c>
       <c r="B75" s="49" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C75" s="45"/>
       <c r="D75" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E75" s="51"/>
     </row>
@@ -6176,11 +7028,11 @@
         <v>69</v>
       </c>
       <c r="B76" s="44" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C76" s="45"/>
       <c r="D76" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E76" s="47"/>
     </row>
@@ -6189,11 +7041,11 @@
         <v>70</v>
       </c>
       <c r="B77" s="49" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C77" s="45"/>
       <c r="D77" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E77" s="51"/>
     </row>
@@ -6202,11 +7054,11 @@
         <v>71</v>
       </c>
       <c r="B78" s="44" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C78" s="45"/>
       <c r="D78" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E78" s="47"/>
     </row>
@@ -6215,11 +7067,11 @@
         <v>72</v>
       </c>
       <c r="B79" s="49" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C79" s="45"/>
       <c r="D79" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E79" s="51"/>
     </row>
@@ -6228,11 +7080,11 @@
         <v>73</v>
       </c>
       <c r="B80" s="44" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C80" s="45"/>
       <c r="D80" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E80" s="47"/>
     </row>
@@ -6241,11 +7093,11 @@
         <v>74</v>
       </c>
       <c r="B81" s="49" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C81" s="45"/>
       <c r="D81" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E81" s="51"/>
     </row>
@@ -6254,11 +7106,11 @@
         <v>75</v>
       </c>
       <c r="B82" s="44" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C82" s="45"/>
       <c r="D82" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E82" s="47"/>
     </row>
@@ -6267,11 +7119,11 @@
         <v>76</v>
       </c>
       <c r="B83" s="49" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C83" s="45"/>
       <c r="D83" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E83" s="51"/>
     </row>
@@ -6280,11 +7132,11 @@
         <v>77</v>
       </c>
       <c r="B84" s="44" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C84" s="45"/>
       <c r="D84" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E84" s="47"/>
     </row>
@@ -6293,11 +7145,11 @@
         <v>78</v>
       </c>
       <c r="B85" s="49" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C85" s="45"/>
       <c r="D85" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E85" s="51"/>
     </row>
@@ -6306,11 +7158,11 @@
         <v>79</v>
       </c>
       <c r="B86" s="44" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C86" s="45"/>
       <c r="D86" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E86" s="47"/>
     </row>
@@ -6319,11 +7171,11 @@
         <v>80</v>
       </c>
       <c r="B87" s="49" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C87" s="45"/>
       <c r="D87" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E87" s="51"/>
     </row>
@@ -6332,11 +7184,11 @@
         <v>81</v>
       </c>
       <c r="B88" s="44" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C88" s="45"/>
       <c r="D88" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E88" s="47"/>
     </row>
@@ -6345,11 +7197,11 @@
         <v>82</v>
       </c>
       <c r="B89" s="49" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C89" s="45"/>
       <c r="D89" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E89" s="51"/>
     </row>
@@ -6358,11 +7210,11 @@
         <v>83</v>
       </c>
       <c r="B90" s="44" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C90" s="45"/>
       <c r="D90" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E90" s="47"/>
     </row>
@@ -6371,11 +7223,11 @@
         <v>84</v>
       </c>
       <c r="B91" s="49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C91" s="45"/>
       <c r="D91" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E91" s="51"/>
     </row>
@@ -6384,11 +7236,11 @@
         <v>85</v>
       </c>
       <c r="B92" s="44" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C92" s="45"/>
       <c r="D92" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E92" s="47"/>
     </row>
@@ -6397,11 +7249,11 @@
         <v>86</v>
       </c>
       <c r="B93" s="49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C93" s="45"/>
       <c r="D93" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E93" s="51"/>
     </row>
@@ -6410,11 +7262,11 @@
         <v>87</v>
       </c>
       <c r="B94" s="44" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C94" s="45"/>
       <c r="D94" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E94" s="47"/>
     </row>
@@ -6423,11 +7275,11 @@
         <v>88</v>
       </c>
       <c r="B95" s="49" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C95" s="45"/>
       <c r="D95" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E95" s="51"/>
     </row>
@@ -6436,11 +7288,11 @@
         <v>89</v>
       </c>
       <c r="B96" s="44" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C96" s="45"/>
       <c r="D96" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E96" s="47"/>
     </row>
@@ -6449,11 +7301,11 @@
         <v>90</v>
       </c>
       <c r="B97" s="49" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C97" s="45"/>
       <c r="D97" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E97" s="51"/>
     </row>
@@ -6462,11 +7314,11 @@
         <v>91</v>
       </c>
       <c r="B98" s="44" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C98" s="45"/>
       <c r="D98" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E98" s="47"/>
     </row>
@@ -6475,11 +7327,11 @@
         <v>92</v>
       </c>
       <c r="B99" s="49" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C99" s="45"/>
       <c r="D99" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E99" s="51"/>
     </row>
@@ -6488,11 +7340,11 @@
         <v>93</v>
       </c>
       <c r="B100" s="44" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C100" s="45"/>
       <c r="D100" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E100" s="47"/>
     </row>
@@ -6501,11 +7353,11 @@
         <v>94</v>
       </c>
       <c r="B101" s="49" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C101" s="45"/>
       <c r="D101" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E101" s="51"/>
     </row>
@@ -6514,11 +7366,11 @@
         <v>95</v>
       </c>
       <c r="B102" s="44" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C102" s="45"/>
       <c r="D102" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E102" s="47"/>
     </row>
@@ -6527,11 +7379,11 @@
         <v>96</v>
       </c>
       <c r="B103" s="49" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C103" s="45"/>
       <c r="D103" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E103" s="51"/>
     </row>
@@ -6540,11 +7392,11 @@
         <v>97</v>
       </c>
       <c r="B104" s="44" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C104" s="45"/>
       <c r="D104" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E104" s="47"/>
     </row>
@@ -6553,11 +7405,11 @@
         <v>98</v>
       </c>
       <c r="B105" s="49" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C105" s="45"/>
       <c r="D105" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E105" s="51"/>
     </row>
@@ -6566,11 +7418,11 @@
         <v>99</v>
       </c>
       <c r="B106" s="44" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C106" s="45"/>
       <c r="D106" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E106" s="47"/>
     </row>
@@ -6579,11 +7431,11 @@
         <v>100</v>
       </c>
       <c r="B107" s="49" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C107" s="45"/>
       <c r="D107" s="50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E107" s="51"/>
     </row>
@@ -6592,11 +7444,11 @@
         <v>101</v>
       </c>
       <c r="B108" s="44" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C108" s="45"/>
       <c r="D108" s="46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E108" s="47"/>
     </row>
@@ -6605,17 +7457,17 @@
         <v>102</v>
       </c>
       <c r="B109" s="59" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C109" s="54"/>
       <c r="D109" s="60" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E109" s="61"/>
     </row>
     <row r="111" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B111" s="57"/>
       <c r="C111" s="57"/>
@@ -6624,7 +7476,7 @@
     </row>
     <row r="113" ht="14" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B113" s="38"/>
       <c r="C113" s="38"/>

</xml_diff>